<commit_message>
feat(catalog): embed product photos in wholesale catalog xlsx
</commit_message>
<xml_diff>
--- a/docs/Oiikon_Wholesale_Catalog_2026-06-24.xlsx
+++ b/docs/Oiikon_Wholesale_Catalog_2026-06-24.xlsx
@@ -28,19 +28,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="22"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <color rgb="00606060"/>
       <sz val="9"/>
     </font>
@@ -144,29 +141,29 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -251,6 +248,236 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -542,18 +769,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -577,51 +805,56 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Photo</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>List Price
 (LA Pickup)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Wholesale
 (+5%)</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>MOQ</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Min. Order
 Value</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
@@ -634,188 +867,193 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>E2000LFP</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>PECRON E2000LFP</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>1,920 Wh</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>2,000 W</t>
         </is>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="F7" s="9" t="n">
         <v>465</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="G7" s="10" t="n">
         <v>488.25</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="H7" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="I7" s="9" t="n">
         <v>11718</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="J7" s="6" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>E3600LFP</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>PECRON E3600LFP</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>3,072 Wh</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>3,600 W</t>
         </is>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="F8" s="14" t="n">
         <v>772</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="G8" s="15" t="n">
         <v>810.6</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="H8" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="H8" s="14" t="n">
+      <c r="I8" s="14" t="n">
         <v>20265</v>
       </c>
-      <c r="I8" s="13" t="n">
+      <c r="J8" s="11" t="n">
         <v>261</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>E3800LFP</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>PECRON E3800LFP</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>3,840 Wh</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>4,200 W</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="F9" s="9" t="n">
         <v>872</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="G9" s="10" t="n">
         <v>915.6</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="H9" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="I9" s="9" t="n">
         <v>22890</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="J9" s="6" t="n">
         <v>400</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>F3000LFP</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>PECRON F3000LFP</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>3,072 Wh</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>3,600 W</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="F10" s="14" t="n">
         <v>595</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="G10" s="15" t="n">
         <v>624.75</v>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="H10" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="I10" s="14" t="n">
         <v>18742.5</v>
       </c>
-      <c r="I10" s="13" t="n">
+      <c r="J10" s="11" t="n">
         <v>853</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>F5000LFP</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>PECRON F5000LFP</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>5,120 Wh</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>7,200 W (120/240V)</t>
         </is>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="F11" s="9" t="n">
         <v>1100</v>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="G11" s="10" t="n">
         <v>1155</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="H11" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="I11" s="9" t="n">
         <v>34650</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="J11" s="6" t="n">
         <v>139</v>
       </c>
     </row>
@@ -826,77 +1064,79 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="13" ht="84" customHeight="1">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>EP3800-48V</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>PECRON EP3800-48V Expansion</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>3,840 Wh</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>48 V — pairs E3800/E3600/F3000/E2400</t>
         </is>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="F13" s="9" t="n">
         <v>490</v>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="G13" s="10" t="n">
         <v>514.5</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="H13" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="I13" s="9" t="n">
         <v>12862.5</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="J13" s="6" t="n">
         <v>600</v>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="14" ht="84" customHeight="1">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>FP5000-48V</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>PECRON FP5000-48V Expansion</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>5,120 Wh</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>48 V — doubles F5000LFP autonomy</t>
         </is>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="F14" s="14" t="n">
         <v>850</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="G14" s="15" t="n">
         <v>892.5</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="H14" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="I14" s="14" t="n">
         <v>21420</v>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="J14" s="11" t="n">
         <v>438</v>
       </c>
     </row>
@@ -907,99 +1147,102 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>PV200</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>PECRON Flexible Monocrystalline 200W</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>200 W</t>
         </is>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="F16" s="9" t="n">
         <v>120</v>
       </c>
-      <c r="F16" s="10" t="n">
+      <c r="G16" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="H16" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="H16" s="9" t="n">
+      <c r="I16" s="9" t="n">
         <v>5040</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="J16" s="6" t="n">
         <v>657</v>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="17" ht="84" customHeight="1">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>PV300</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>PECRON Flexible Monocrystalline 300W</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>300 W</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="F17" s="14" t="n">
         <v>180</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="G17" s="15" t="n">
         <v>189</v>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="H17" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="H17" s="14" t="n">
+      <c r="I17" s="14" t="n">
         <v>6237</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="J17" s="11" t="n">
         <v>171</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Notes:  Wholesale price = List Price (LA pickup) + 5% margin.  MOQ = Minimum Order Quantity per model.  Min. Order Value = Wholesale Price × MOQ.  Stock subject to prior sale — confirm availability at time of order.  Specs per Oiikon PECRON catalog.</t>
+          <t>Notes:  Wholesale price = List Price (LA pickup) + 5% margin.  MOQ = Minimum Order Quantity per model.  Min. Order Value = Wholesale Price × MOQ.  Stock subject to prior sale — confirm availability at time of order.  Product images &amp; specs per Oiikon PECRON catalog.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A19:J19"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(catalog): add Sale Price (retail) column derived from profit margins
</commit_message>
<xml_diff>
--- a/docs/Oiikon_Wholesale_Catalog_2026-06-24.xlsx
+++ b/docs/Oiikon_Wholesale_Catalog_2026-06-24.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,10 @@
     <font>
       <b val="1"/>
       <color rgb="002E5496"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
     </font>
     <font>
       <i val="1"/>
@@ -124,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -156,6 +160,9 @@
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -171,7 +178,10 @@
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -769,19 +779,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -845,16 +856,22 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
+          <t>Sale Price
+(Retail)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
           <t>MOQ</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Min. Order
 Value</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
@@ -895,51 +912,57 @@
       <c r="G7" s="10" t="n">
         <v>488.25</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="H7" s="11" t="n">
+        <v>599</v>
+      </c>
+      <c r="I7" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="J7" s="9" t="n">
         <v>11718</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="K7" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="8" ht="84" customHeight="1">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>E3600LFP</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>PECRON E3600LFP</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>3,072 Wh</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>3,600 W</t>
         </is>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="15" t="n">
         <v>772</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="16" t="n">
         <v>810.6</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="17" t="n">
+        <v>1103</v>
+      </c>
+      <c r="I8" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="J8" s="15" t="n">
         <v>20265</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="K8" s="12" t="n">
         <v>261</v>
       </c>
     </row>
@@ -971,51 +994,57 @@
       <c r="G9" s="10" t="n">
         <v>915.6</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="11" t="n">
+        <v>1195</v>
+      </c>
+      <c r="I9" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="I9" s="9" t="n">
+      <c r="J9" s="9" t="n">
         <v>22890</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="K9" s="6" t="n">
         <v>400</v>
       </c>
     </row>
     <row r="10" ht="84" customHeight="1">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>F3000LFP</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>PECRON F3000LFP</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>3,072 Wh</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>3,600 W</t>
         </is>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="15" t="n">
         <v>595</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="16" t="n">
         <v>624.75</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="17" t="n">
+        <v>849</v>
+      </c>
+      <c r="I10" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="I10" s="14" t="n">
+      <c r="J10" s="15" t="n">
         <v>18742.5</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="K10" s="12" t="n">
         <v>853</v>
       </c>
     </row>
@@ -1047,13 +1076,16 @@
       <c r="G11" s="10" t="n">
         <v>1155</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="11" t="n">
+        <v>1999</v>
+      </c>
+      <c r="I11" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="J11" s="9" t="n">
         <v>34650</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>139</v>
       </c>
     </row>
@@ -1092,51 +1124,57 @@
       <c r="G13" s="10" t="n">
         <v>514.5</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="11" t="n">
+        <v>721</v>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="I13" s="9" t="n">
+      <c r="J13" s="9" t="n">
         <v>12862.5</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="K13" s="6" t="n">
         <v>600</v>
       </c>
     </row>
     <row r="14" ht="84" customHeight="1">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>FP5000-48V</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>PECRON FP5000-48V Expansion</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>5,120 Wh</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>48 V — doubles F5000LFP autonomy</t>
         </is>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="15" t="n">
         <v>850</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="16" t="n">
         <v>892.5</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="17" t="n">
+        <v>1299</v>
+      </c>
+      <c r="I14" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="J14" s="15" t="n">
         <v>21420</v>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="K14" s="12" t="n">
         <v>438</v>
       </c>
     </row>
@@ -1175,56 +1213,62 @@
       <c r="G16" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="I16" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="J16" s="9" t="n">
         <v>5040</v>
       </c>
-      <c r="J16" s="6" t="n">
+      <c r="K16" s="6" t="n">
         <v>657</v>
       </c>
     </row>
     <row r="17" ht="84" customHeight="1">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>PV300</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>PECRON Flexible Monocrystalline 300W</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>300 W</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="15" t="n">
         <v>180</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="16" t="n">
         <v>189</v>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H17" s="17" t="n">
+        <v>273</v>
+      </c>
+      <c r="I17" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="I17" s="14" t="n">
+      <c r="J17" s="15" t="n">
         <v>6237</v>
       </c>
-      <c r="J17" s="11" t="n">
+      <c r="K17" s="12" t="n">
         <v>171</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Notes:  Wholesale price = List Price (LA pickup) + 5% margin.  MOQ = Minimum Order Quantity per model.  Min. Order Value = Wholesale Price × MOQ.  Stock subject to prior sale — confirm availability at time of order.  Product images &amp; specs per Oiikon PECRON catalog.</t>
         </is>
@@ -1232,13 +1276,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>